<commit_message>
Updated Description, Outcome Message and added Output Variable LBTOX
</commit_message>
<xml_diff>
--- a/rules/CORE-000169/negative/01/data/unit-test-coreid-CG185-negative.xlsx
+++ b/rules/CORE-000169/negative/01/data/unit-test-coreid-CG185-negative.xlsx
@@ -36,7 +36,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -53,12 +53,15 @@
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
       <i/>
     </font>
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
-      <i/>
     </font>
     <font>
       <sz val="11"/>
@@ -84,7 +87,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFFCC"/>
+        <fgColor rgb="FFFFFF00"/>
         <bgColor/>
       </patternFill>
     </fill>
@@ -119,10 +122,10 @@
     <xf numFmtId="0" fontId="1" fillId="1" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -465,10 +468,10 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="str">
+      <c r="A2" s="4" t="str">
         <v>sdtmig</v>
       </c>
-      <c r="B2" s="2" t="str">
+      <c r="B2" s="4" t="str">
         <v>3-4</v>
       </c>
     </row>
@@ -492,10 +495,10 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="str">
+      <c r="A2" s="4" t="str">
         <v>lb.xpt</v>
       </c>
-      <c r="B2" s="2" t="str">
+      <c r="B2" s="4" t="str">
         <v>Labotory Results</v>
       </c>
     </row>
@@ -508,7 +511,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F3"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="str">
@@ -531,28 +534,48 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2">
+      <c r="A2" s="4">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="str">
+      <c r="B2" s="4" t="str">
         <v>lb.xpt</v>
       </c>
-      <c r="C2" s="2" t="str">
+      <c r="C2" s="4" t="str">
         <v>Record</v>
       </c>
-      <c r="D2" s="2">
+      <c r="D2" s="4">
         <v>5</v>
       </c>
-      <c r="E2" s="2" t="str">
+      <c r="E2" s="4" t="str">
         <v>LBTOXGR</v>
       </c>
-      <c r="F2" s="2" t="str">
+      <c r="F2" s="4" t="str">
+        <v>Grade 2</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2">
+        <v>1</v>
+      </c>
+      <c r="B3" s="2" t="str">
+        <v>lb.xpt</v>
+      </c>
+      <c r="C3" s="2" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D3" s="2">
+        <v>5</v>
+      </c>
+      <c r="E3" s="2" t="str">
+        <v>LBTOX</v>
+      </c>
+      <c r="F3" s="2" t="str">
         <v>Grade 2</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F3"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -639,13 +662,13 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="str">
+      <c r="A2" s="5" t="str">
         <v>Study Identifier</v>
       </c>
-      <c r="B2" s="4" t="str">
+      <c r="B2" s="5" t="str">
         <v>Domain Abbreviation</v>
       </c>
-      <c r="C2" s="4" t="str">
+      <c r="C2" s="5" t="str">
         <v>Unique Subject Identifier</v>
       </c>
       <c r="D2" s="5" t="str">
@@ -870,310 +893,310 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="str">
+      <c r="A5" s="4" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B5" s="6" t="str">
+      <c r="B5" s="4" t="str">
         <v>LB</v>
       </c>
-      <c r="C5" s="6" t="str">
+      <c r="C5" s="4" t="str">
         <v>CDISC001</v>
       </c>
-      <c r="D5" s="6">
+      <c r="D5" s="4">
         <v>1</v>
       </c>
-      <c r="E5" s="6" t="str">
+      <c r="E5" s="4" t="str">
         <v>ALB</v>
       </c>
-      <c r="F5" s="6" t="str">
+      <c r="F5" s="4" t="str">
         <v>Albumin</v>
       </c>
-      <c r="G5" s="6" t="str">
+      <c r="G5" s="4" t="str">
         <v>CHEMISTRY</v>
       </c>
-      <c r="H5" s="6" t="str">
+      <c r="H5" s="4" t="str">
         <v>3.9</v>
       </c>
-      <c r="I5" s="6" t="str">
+      <c r="I5" s="4" t="str">
         <v>g/dL</v>
       </c>
-      <c r="J5" s="6" t="str">
+      <c r="J5" s="4" t="str">
         <v>3.5</v>
       </c>
-      <c r="K5" s="6" t="str">
+      <c r="K5" s="4" t="str">
         <v>4.6</v>
       </c>
-      <c r="L5" s="6" t="str">
+      <c r="L5" s="4" t="str">
         <v>39</v>
       </c>
-      <c r="M5" s="6">
+      <c r="M5" s="4">
         <v>39</v>
       </c>
-      <c r="N5" s="6" t="str">
+      <c r="N5" s="4" t="str">
         <v>g/L</v>
       </c>
-      <c r="O5" s="6">
+      <c r="O5" s="4">
         <v>35</v>
       </c>
-      <c r="P5" s="6">
+      <c r="P5" s="4">
         <v>46</v>
       </c>
-      <c r="Q5" s="6" t="str">
+      <c r="Q5" s="4" t="str">
         <v>NORMAL</v>
       </c>
-      <c r="R5" s="6" t="str">
+      <c r="R5" s="4" t="str">
         <v>Y</v>
       </c>
-      <c r="S5" s="6">
+      <c r="S5" s="4">
         <v>1</v>
       </c>
-      <c r="T5" s="6" t="str">
+      <c r="T5" s="4" t="str">
         <v>SCREENING 1</v>
       </c>
-      <c r="U5" s="6" t="str">
+      <c r="U5" s="4" t="str">
         <v>SCREENING</v>
       </c>
-      <c r="V5" s="6" t="str">
+      <c r="V5" s="4" t="str">
         <v>2012-11-23T11:20</v>
       </c>
-      <c r="W5" s="6">
+      <c r="W5" s="4">
         <v>-7</v>
       </c>
-      <c r="X5" s="2" t="str">
-        <v/>
+      <c r="X5" s="6" t="str">
+        <v>Grade 2</v>
       </c>
       <c r="Y5" s="7" t="str">
         <v>Grade 2</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="str">
+      <c r="A6" s="4" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B6" s="6" t="str">
+      <c r="B6" s="4" t="str">
         <v>LB</v>
       </c>
-      <c r="C6" s="6" t="str">
+      <c r="C6" s="4" t="str">
         <v>CDISC001</v>
       </c>
-      <c r="D6" s="6">
+      <c r="D6" s="4">
         <v>2</v>
       </c>
-      <c r="E6" s="6" t="str">
+      <c r="E6" s="4" t="str">
         <v>ALP</v>
       </c>
-      <c r="F6" s="6" t="str">
+      <c r="F6" s="4" t="str">
         <v>Alkaline Phosphatase</v>
       </c>
-      <c r="G6" s="6" t="str">
+      <c r="G6" s="4" t="str">
         <v>CHEMISTRY</v>
       </c>
-      <c r="H6" s="6" t="str">
+      <c r="H6" s="4" t="str">
         <v>93</v>
       </c>
-      <c r="I6" s="6" t="str">
+      <c r="I6" s="4" t="str">
         <v>U/L</v>
       </c>
-      <c r="J6" s="6" t="str">
+      <c r="J6" s="4" t="str">
         <v>35</v>
       </c>
-      <c r="K6" s="6" t="str">
+      <c r="K6" s="4" t="str">
         <v>115</v>
       </c>
-      <c r="L6" s="6" t="str">
+      <c r="L6" s="4" t="str">
         <v>93</v>
       </c>
-      <c r="M6" s="6">
+      <c r="M6" s="4">
         <v>93</v>
       </c>
-      <c r="N6" s="6" t="str">
+      <c r="N6" s="4" t="str">
         <v>U/L</v>
       </c>
-      <c r="O6" s="6">
+      <c r="O6" s="4">
         <v>35</v>
       </c>
-      <c r="P6" s="6">
+      <c r="P6" s="4">
         <v>115</v>
       </c>
-      <c r="Q6" s="6" t="str">
+      <c r="Q6" s="4" t="str">
         <v>NORMAL</v>
       </c>
-      <c r="R6" s="6" t="str">
+      <c r="R6" s="4" t="str">
         <v>Y</v>
       </c>
-      <c r="S6" s="6">
+      <c r="S6" s="4">
         <v>1</v>
       </c>
-      <c r="T6" s="6" t="str">
+      <c r="T6" s="4" t="str">
         <v>SCREENING 1</v>
       </c>
-      <c r="U6" s="6" t="str">
+      <c r="U6" s="4" t="str">
         <v>SCREENING</v>
       </c>
-      <c r="V6" s="6" t="str">
+      <c r="V6" s="4" t="str">
         <v>2012-11-23T11:20</v>
       </c>
-      <c r="W6" s="6">
+      <c r="W6" s="4">
         <v>-7</v>
       </c>
-      <c r="X6" s="2" t="str">
+      <c r="X6" s="4" t="str">
         <v/>
       </c>
-      <c r="Y6" s="2">
+      <c r="Y6" s="4">
         <v>2</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="str">
+      <c r="A7" s="4" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B7" s="6" t="str">
+      <c r="B7" s="4" t="str">
         <v>LB</v>
       </c>
-      <c r="C7" s="6" t="str">
+      <c r="C7" s="4" t="str">
         <v>CDISC001</v>
       </c>
-      <c r="D7" s="6">
+      <c r="D7" s="4">
         <v>2</v>
       </c>
-      <c r="E7" s="6" t="str">
+      <c r="E7" s="4" t="str">
         <v>ALP</v>
       </c>
-      <c r="F7" s="6" t="str">
+      <c r="F7" s="4" t="str">
         <v>Alkaline Phosphatase</v>
       </c>
-      <c r="G7" s="6" t="str">
+      <c r="G7" s="4" t="str">
         <v>CHEMISTRY</v>
       </c>
-      <c r="H7" s="6" t="str">
+      <c r="H7" s="4" t="str">
         <v>93</v>
       </c>
-      <c r="I7" s="6" t="str">
+      <c r="I7" s="4" t="str">
         <v>U/L</v>
       </c>
-      <c r="J7" s="6" t="str">
+      <c r="J7" s="4" t="str">
         <v>35</v>
       </c>
-      <c r="K7" s="6" t="str">
+      <c r="K7" s="4" t="str">
         <v>115</v>
       </c>
-      <c r="L7" s="6" t="str">
+      <c r="L7" s="4" t="str">
         <v>93</v>
       </c>
-      <c r="M7" s="6">
+      <c r="M7" s="4">
         <v>93</v>
       </c>
-      <c r="N7" s="6" t="str">
+      <c r="N7" s="4" t="str">
         <v>U/L</v>
       </c>
-      <c r="O7" s="6">
+      <c r="O7" s="4">
         <v>35</v>
       </c>
-      <c r="P7" s="6">
+      <c r="P7" s="4">
         <v>115</v>
       </c>
-      <c r="Q7" s="6" t="str">
+      <c r="Q7" s="4" t="str">
         <v>NORMAL</v>
       </c>
-      <c r="R7" s="6" t="str">
+      <c r="R7" s="4" t="str">
         <v>Y</v>
       </c>
-      <c r="S7" s="6">
+      <c r="S7" s="4">
         <v>1</v>
       </c>
-      <c r="T7" s="6" t="str">
+      <c r="T7" s="4" t="str">
         <v>SCREENING 1</v>
       </c>
-      <c r="U7" s="6" t="str">
+      <c r="U7" s="4" t="str">
         <v>SCREENING</v>
       </c>
-      <c r="V7" s="6" t="str">
+      <c r="V7" s="4" t="str">
         <v>2012-11-23T11:20</v>
       </c>
-      <c r="W7" s="6">
+      <c r="W7" s="4">
         <v>-7</v>
       </c>
-      <c r="X7" s="2" t="str">
+      <c r="X7" s="4" t="str">
         <v/>
       </c>
-      <c r="Y7" s="2" t="str">
+      <c r="Y7" s="4" t="str">
         <v>Grade II</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="str">
+      <c r="A8" s="4" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B8" s="6" t="str">
+      <c r="B8" s="4" t="str">
         <v>LB</v>
       </c>
-      <c r="C8" s="6" t="str">
+      <c r="C8" s="4" t="str">
         <v>CDISC002</v>
       </c>
-      <c r="D8" s="6">
+      <c r="D8" s="4">
         <v>1</v>
       </c>
-      <c r="E8" s="6" t="str">
+      <c r="E8" s="4" t="str">
         <v>ALB</v>
       </c>
-      <c r="F8" s="6" t="str">
+      <c r="F8" s="4" t="str">
         <v>Albumin</v>
       </c>
-      <c r="G8" s="6" t="str">
+      <c r="G8" s="4" t="str">
         <v>CHEMISTRY</v>
       </c>
-      <c r="H8" s="6" t="str">
+      <c r="H8" s="4" t="str">
         <v>3.9</v>
       </c>
-      <c r="I8" s="6" t="str">
+      <c r="I8" s="4" t="str">
         <v>g/dL</v>
       </c>
-      <c r="J8" s="6" t="str">
+      <c r="J8" s="4" t="str">
         <v>3.5</v>
       </c>
-      <c r="K8" s="6" t="str">
+      <c r="K8" s="4" t="str">
         <v>4.6</v>
       </c>
-      <c r="L8" s="6" t="str">
+      <c r="L8" s="4" t="str">
         <v>39</v>
       </c>
-      <c r="M8" s="6">
+      <c r="M8" s="4">
         <v>39</v>
       </c>
-      <c r="N8" s="6" t="str">
+      <c r="N8" s="4" t="str">
         <v>g/L</v>
       </c>
-      <c r="O8" s="6">
+      <c r="O8" s="4">
         <v>35</v>
       </c>
-      <c r="P8" s="6">
+      <c r="P8" s="4">
         <v>46</v>
       </c>
-      <c r="Q8" s="6" t="str">
+      <c r="Q8" s="4" t="str">
         <v>NORMAL</v>
       </c>
-      <c r="R8" s="6" t="str">
+      <c r="R8" s="4" t="str">
         <v>Y</v>
       </c>
-      <c r="S8" s="6">
+      <c r="S8" s="4">
         <v>1</v>
       </c>
-      <c r="T8" s="6" t="str">
+      <c r="T8" s="4" t="str">
         <v>SCREENING 1</v>
       </c>
-      <c r="U8" s="6" t="str">
+      <c r="U8" s="4" t="str">
         <v>SCREENING</v>
       </c>
-      <c r="V8" s="6" t="str">
+      <c r="V8" s="4" t="str">
         <v>2012-11-23T11:20</v>
       </c>
-      <c r="W8" s="6">
+      <c r="W8" s="4">
         <v>-7</v>
       </c>
-      <c r="X8" s="2" t="str">
+      <c r="X8" s="4" t="str">
         <v/>
       </c>
-      <c r="Y8" s="2">
+      <c r="Y8" s="4">
         <v>4</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Fixed Outcome.Message text; Executability is now Partially Executable - Possible Overreporting.
</commit_message>
<xml_diff>
--- a/rules/CORE-000169/negative/01/data/unit-test-coreid-CG185-negative.xlsx
+++ b/rules/CORE-000169/negative/01/data/unit-test-coreid-CG185-negative.xlsx
@@ -36,7 +36,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -48,16 +48,6 @@
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <i/>
     </font>
     <font>
       <sz val="11"/>
@@ -68,7 +58,7 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none">
         <bgColor/>
@@ -81,19 +71,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFFCC"/>
+        <fgColor rgb="FFffffcc"/>
         <bgColor/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
+        <fgColor rgb="FFffff00"/>
         <bgColor/>
       </patternFill>
     </fill>
@@ -117,15 +101,13 @@
   <cellStyleXfs>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="1" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -468,10 +450,10 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="str">
+      <c r="A2" s="3" t="str">
         <v>sdtmig</v>
       </c>
-      <c r="B2" s="4" t="str">
+      <c r="B2" s="3" t="str">
         <v>3-4</v>
       </c>
     </row>
@@ -495,10 +477,10 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="str">
+      <c r="A2" s="3" t="str">
         <v>lb.xpt</v>
       </c>
-      <c r="B2" s="4" t="str">
+      <c r="B2" s="3" t="str">
         <v>Labotory Results</v>
       </c>
     </row>
@@ -511,7 +493,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F7"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="str">
@@ -534,48 +516,128 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4">
+      <c r="A2" s="3">
         <v>1</v>
       </c>
-      <c r="B2" s="4" t="str">
+      <c r="B2" s="3" t="str">
         <v>lb.xpt</v>
       </c>
-      <c r="C2" s="4" t="str">
+      <c r="C2" s="3" t="str">
         <v>Record</v>
       </c>
-      <c r="D2" s="4">
+      <c r="D2" s="3">
         <v>5</v>
       </c>
-      <c r="E2" s="4" t="str">
+      <c r="E2" s="3" t="str">
         <v>LBTOXGR</v>
       </c>
-      <c r="F2" s="4" t="str">
+      <c r="F2" s="3" t="str">
         <v>Grade 2</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2">
+      <c r="A3" s="3">
         <v>1</v>
       </c>
-      <c r="B3" s="2" t="str">
+      <c r="B3" s="3" t="str">
         <v>lb.xpt</v>
       </c>
-      <c r="C3" s="2" t="str">
+      <c r="C3" s="3" t="str">
         <v>Record</v>
       </c>
-      <c r="D3" s="2">
+      <c r="D3" s="3">
         <v>5</v>
       </c>
-      <c r="E3" s="2" t="str">
+      <c r="E3" s="3" t="str">
         <v>LBTOX</v>
       </c>
-      <c r="F3" s="2" t="str">
+      <c r="F3" s="3" t="str">
         <v>Grade 2</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3">
+        <v>1</v>
+      </c>
+      <c r="B4" s="3" t="str">
+        <v>lb.xpt</v>
+      </c>
+      <c r="C4" s="3" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D4" s="3">
+        <v>5</v>
+      </c>
+      <c r="E4" s="3" t="str">
+        <v>LBTESTCD</v>
+      </c>
+      <c r="F4" s="3" t="str">
+        <v>ALB</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="str">
+        <v/>
+      </c>
+      <c r="B5" s="3" t="str">
+        <v/>
+      </c>
+      <c r="C5" s="3" t="str">
+        <v/>
+      </c>
+      <c r="D5" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E5" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F5" s="3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="str">
+        <v/>
+      </c>
+      <c r="B6" s="3" t="str">
+        <v/>
+      </c>
+      <c r="C6" s="3" t="str">
+        <v/>
+      </c>
+      <c r="D6" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E6" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F6" s="3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="str">
+        <v/>
+      </c>
+      <c r="B7" s="3" t="str">
+        <v/>
+      </c>
+      <c r="C7" s="3" t="str">
+        <v/>
+      </c>
+      <c r="D7" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E7" s="3" t="str">
+        <v/>
+      </c>
+      <c r="F7" s="3" t="str">
+        <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F7"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -662,541 +724,541 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="str">
+      <c r="A2" s="4" t="str">
         <v>Study Identifier</v>
       </c>
-      <c r="B2" s="5" t="str">
+      <c r="B2" s="4" t="str">
         <v>Domain Abbreviation</v>
       </c>
-      <c r="C2" s="5" t="str">
+      <c r="C2" s="4" t="str">
         <v>Unique Subject Identifier</v>
       </c>
-      <c r="D2" s="5" t="str">
+      <c r="D2" s="4" t="str">
         <v>Sequence Number</v>
       </c>
-      <c r="E2" s="5" t="str">
+      <c r="E2" s="4" t="str">
         <v>Lab Test or Examination Short Name</v>
       </c>
-      <c r="F2" s="5" t="str">
+      <c r="F2" s="4" t="str">
         <v>Lab Test or Examination Name</v>
       </c>
-      <c r="G2" s="5" t="str">
+      <c r="G2" s="4" t="str">
         <v>Category for Lab Test</v>
       </c>
-      <c r="H2" s="5" t="str">
+      <c r="H2" s="4" t="str">
         <v>Result or Finding in Original Units</v>
       </c>
-      <c r="I2" s="5" t="str">
+      <c r="I2" s="4" t="str">
         <v>Original Units</v>
       </c>
-      <c r="J2" s="5" t="str">
+      <c r="J2" s="4" t="str">
         <v>Reference Range Lower Limit in Orig Unit</v>
       </c>
-      <c r="K2" s="5" t="str">
+      <c r="K2" s="4" t="str">
         <v>Reference Range Upper Limit in Orig Unit</v>
       </c>
-      <c r="L2" s="5" t="str">
+      <c r="L2" s="4" t="str">
         <v>Character Result/Finding in Std Format</v>
       </c>
-      <c r="M2" s="5" t="str">
+      <c r="M2" s="4" t="str">
         <v>Numeric Result/Finding in Standard Units</v>
       </c>
-      <c r="N2" s="5" t="str">
+      <c r="N2" s="4" t="str">
         <v>Standard Units</v>
       </c>
-      <c r="O2" s="5" t="str">
+      <c r="O2" s="4" t="str">
         <v>Reference Range Lower Limit-Std Units</v>
       </c>
-      <c r="P2" s="5" t="str">
+      <c r="P2" s="4" t="str">
         <v>Reference Range Upper Limit-Std Units</v>
       </c>
-      <c r="Q2" s="5" t="str">
+      <c r="Q2" s="4" t="str">
         <v>Reference Range Indicator</v>
       </c>
-      <c r="R2" s="5" t="str">
+      <c r="R2" s="4" t="str">
         <v>Last Observation Before Exposure Flag</v>
       </c>
-      <c r="S2" s="5" t="str">
+      <c r="S2" s="4" t="str">
         <v>Visit Number</v>
       </c>
-      <c r="T2" s="5" t="str">
+      <c r="T2" s="4" t="str">
         <v>Visit Name</v>
       </c>
-      <c r="U2" s="5" t="str">
+      <c r="U2" s="4" t="str">
         <v>Epoch</v>
       </c>
-      <c r="V2" s="5" t="str">
+      <c r="V2" s="4" t="str">
         <v>Date/Time of Specimen Collection</v>
       </c>
-      <c r="W2" s="5" t="str">
+      <c r="W2" s="4" t="str">
         <v>Study Day of Specimen Collection</v>
       </c>
-      <c r="X2" s="5" t="str">
+      <c r="X2" s="4" t="str">
         <v>Toxicity</v>
       </c>
-      <c r="Y2" s="5" t="str">
+      <c r="Y2" s="4" t="str">
         <v>Standard Toxicity Grade</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="B3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="C3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="D3" s="5" t="str">
+      <c r="A3" s="4" t="str">
+        <v>Char</v>
+      </c>
+      <c r="B3" s="4" t="str">
+        <v>Char</v>
+      </c>
+      <c r="C3" s="4" t="str">
+        <v>Char</v>
+      </c>
+      <c r="D3" s="4" t="str">
         <v>Num</v>
       </c>
-      <c r="E3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="F3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="G3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="H3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="I3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="J3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="K3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="L3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="M3" s="5" t="str">
+      <c r="E3" s="4" t="str">
+        <v>Char</v>
+      </c>
+      <c r="F3" s="4" t="str">
+        <v>Char</v>
+      </c>
+      <c r="G3" s="4" t="str">
+        <v>Char</v>
+      </c>
+      <c r="H3" s="4" t="str">
+        <v>Char</v>
+      </c>
+      <c r="I3" s="4" t="str">
+        <v>Char</v>
+      </c>
+      <c r="J3" s="4" t="str">
+        <v>Char</v>
+      </c>
+      <c r="K3" s="4" t="str">
+        <v>Char</v>
+      </c>
+      <c r="L3" s="4" t="str">
+        <v>Char</v>
+      </c>
+      <c r="M3" s="4" t="str">
         <v>Num</v>
       </c>
-      <c r="N3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="O3" s="5" t="str">
+      <c r="N3" s="4" t="str">
+        <v>Char</v>
+      </c>
+      <c r="O3" s="4" t="str">
         <v>Num</v>
       </c>
-      <c r="P3" s="5" t="str">
+      <c r="P3" s="4" t="str">
         <v>Num</v>
       </c>
-      <c r="Q3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="R3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="S3" s="5" t="str">
+      <c r="Q3" s="4" t="str">
+        <v>Char</v>
+      </c>
+      <c r="R3" s="4" t="str">
+        <v>Char</v>
+      </c>
+      <c r="S3" s="4" t="str">
         <v>Num</v>
       </c>
-      <c r="T3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="U3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="V3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="W3" s="5" t="str">
+      <c r="T3" s="4" t="str">
+        <v>Char</v>
+      </c>
+      <c r="U3" s="4" t="str">
+        <v>Char</v>
+      </c>
+      <c r="V3" s="4" t="str">
+        <v>Char</v>
+      </c>
+      <c r="W3" s="4" t="str">
         <v>Num</v>
       </c>
-      <c r="X3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="Y3" s="5" t="str">
+      <c r="X3" s="4" t="str">
+        <v>Char</v>
+      </c>
+      <c r="Y3" s="4" t="str">
         <v>Char</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5">
+      <c r="A4" s="4">
         <v>12</v>
       </c>
-      <c r="B4" s="5">
+      <c r="B4" s="4">
         <v>2</v>
       </c>
-      <c r="C4" s="5">
+      <c r="C4" s="4">
         <v>8</v>
       </c>
-      <c r="D4" s="5">
+      <c r="D4" s="4">
         <v>8</v>
       </c>
-      <c r="E4" s="5">
+      <c r="E4" s="4">
         <v>7</v>
       </c>
-      <c r="F4" s="5">
+      <c r="F4" s="4">
         <v>39</v>
       </c>
-      <c r="G4" s="5">
+      <c r="G4" s="4">
         <v>10</v>
       </c>
-      <c r="H4" s="5">
+      <c r="H4" s="4">
         <v>6</v>
       </c>
-      <c r="I4" s="5">
+      <c r="I4" s="4">
         <v>7</v>
       </c>
-      <c r="J4" s="5">
+      <c r="J4" s="4">
         <v>200</v>
       </c>
-      <c r="K4" s="5">
+      <c r="K4" s="4">
         <v>200</v>
       </c>
-      <c r="L4" s="5">
+      <c r="L4" s="4">
         <v>8</v>
       </c>
-      <c r="M4" s="5">
+      <c r="M4" s="4">
         <v>8</v>
       </c>
-      <c r="N4" s="5">
+      <c r="N4" s="4">
         <v>7</v>
       </c>
-      <c r="O4" s="5">
+      <c r="O4" s="4">
         <v>8</v>
       </c>
-      <c r="P4" s="5">
+      <c r="P4" s="4">
         <v>8</v>
       </c>
-      <c r="Q4" s="5">
+      <c r="Q4" s="4">
         <v>8</v>
       </c>
-      <c r="R4" s="5">
+      <c r="R4" s="4">
         <v>1</v>
       </c>
-      <c r="S4" s="5">
+      <c r="S4" s="4">
         <v>8</v>
       </c>
-      <c r="T4" s="5">
+      <c r="T4" s="4">
         <v>200</v>
       </c>
-      <c r="U4" s="5">
+      <c r="U4" s="4">
         <v>9</v>
       </c>
-      <c r="V4" s="5">
+      <c r="V4" s="4">
         <v>19</v>
       </c>
-      <c r="W4" s="5">
+      <c r="W4" s="4">
         <v>8</v>
       </c>
-      <c r="X4" s="5">
+      <c r="X4" s="4">
         <v>50</v>
       </c>
-      <c r="Y4" s="5">
+      <c r="Y4" s="4">
         <v>50</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="str">
+      <c r="A5" s="3" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B5" s="4" t="str">
+      <c r="B5" s="3" t="str">
         <v>LB</v>
       </c>
-      <c r="C5" s="4" t="str">
+      <c r="C5" s="3" t="str">
         <v>CDISC001</v>
       </c>
-      <c r="D5" s="4">
+      <c r="D5" s="3">
         <v>1</v>
       </c>
-      <c r="E5" s="4" t="str">
+      <c r="E5" s="5" t="str">
         <v>ALB</v>
       </c>
-      <c r="F5" s="4" t="str">
+      <c r="F5" s="3" t="str">
         <v>Albumin</v>
       </c>
-      <c r="G5" s="4" t="str">
+      <c r="G5" s="3" t="str">
         <v>CHEMISTRY</v>
       </c>
-      <c r="H5" s="4" t="str">
+      <c r="H5" s="3">
         <v>3.9</v>
       </c>
-      <c r="I5" s="4" t="str">
+      <c r="I5" s="3" t="str">
         <v>g/dL</v>
       </c>
-      <c r="J5" s="4" t="str">
+      <c r="J5" s="3">
         <v>3.5</v>
       </c>
-      <c r="K5" s="4" t="str">
+      <c r="K5" s="3">
         <v>4.6</v>
       </c>
-      <c r="L5" s="4" t="str">
+      <c r="L5" s="3">
         <v>39</v>
       </c>
-      <c r="M5" s="4">
+      <c r="M5" s="3">
         <v>39</v>
       </c>
-      <c r="N5" s="4" t="str">
+      <c r="N5" s="3" t="str">
         <v>g/L</v>
       </c>
-      <c r="O5" s="4">
+      <c r="O5" s="3">
         <v>35</v>
       </c>
-      <c r="P5" s="4">
+      <c r="P5" s="3">
         <v>46</v>
       </c>
-      <c r="Q5" s="4" t="str">
+      <c r="Q5" s="3" t="str">
         <v>NORMAL</v>
       </c>
-      <c r="R5" s="4" t="str">
+      <c r="R5" s="3" t="str">
         <v>Y</v>
       </c>
-      <c r="S5" s="4">
+      <c r="S5" s="3">
         <v>1</v>
       </c>
-      <c r="T5" s="4" t="str">
+      <c r="T5" s="3" t="str">
         <v>SCREENING 1</v>
       </c>
-      <c r="U5" s="4" t="str">
+      <c r="U5" s="3" t="str">
         <v>SCREENING</v>
       </c>
-      <c r="V5" s="4" t="str">
+      <c r="V5" s="3" t="str">
         <v>2012-11-23T11:20</v>
       </c>
-      <c r="W5" s="4">
+      <c r="W5" s="3">
         <v>-7</v>
       </c>
-      <c r="X5" s="6" t="str">
+      <c r="X5" s="5" t="str">
         <v>Grade 2</v>
       </c>
-      <c r="Y5" s="7" t="str">
+      <c r="Y5" s="5" t="str">
         <v>Grade 2</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="str">
+      <c r="A6" s="3" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B6" s="4" t="str">
+      <c r="B6" s="3" t="str">
         <v>LB</v>
       </c>
-      <c r="C6" s="4" t="str">
+      <c r="C6" s="3" t="str">
         <v>CDISC001</v>
       </c>
-      <c r="D6" s="4">
+      <c r="D6" s="3">
         <v>2</v>
       </c>
-      <c r="E6" s="4" t="str">
+      <c r="E6" s="3" t="str">
         <v>ALP</v>
       </c>
-      <c r="F6" s="4" t="str">
+      <c r="F6" s="3" t="str">
         <v>Alkaline Phosphatase</v>
       </c>
-      <c r="G6" s="4" t="str">
+      <c r="G6" s="3" t="str">
         <v>CHEMISTRY</v>
       </c>
-      <c r="H6" s="4" t="str">
+      <c r="H6" s="3">
         <v>93</v>
       </c>
-      <c r="I6" s="4" t="str">
+      <c r="I6" s="3" t="str">
         <v>U/L</v>
       </c>
-      <c r="J6" s="4" t="str">
+      <c r="J6" s="3">
         <v>35</v>
       </c>
-      <c r="K6" s="4" t="str">
+      <c r="K6" s="3">
         <v>115</v>
       </c>
-      <c r="L6" s="4" t="str">
+      <c r="L6" s="3">
         <v>93</v>
       </c>
-      <c r="M6" s="4">
+      <c r="M6" s="3">
         <v>93</v>
       </c>
-      <c r="N6" s="4" t="str">
+      <c r="N6" s="3" t="str">
         <v>U/L</v>
       </c>
-      <c r="O6" s="4">
+      <c r="O6" s="3">
         <v>35</v>
       </c>
-      <c r="P6" s="4">
+      <c r="P6" s="3">
         <v>115</v>
       </c>
-      <c r="Q6" s="4" t="str">
+      <c r="Q6" s="3" t="str">
         <v>NORMAL</v>
       </c>
-      <c r="R6" s="4" t="str">
+      <c r="R6" s="3" t="str">
         <v>Y</v>
       </c>
-      <c r="S6" s="4">
+      <c r="S6" s="3">
         <v>1</v>
       </c>
-      <c r="T6" s="4" t="str">
+      <c r="T6" s="3" t="str">
         <v>SCREENING 1</v>
       </c>
-      <c r="U6" s="4" t="str">
+      <c r="U6" s="3" t="str">
         <v>SCREENING</v>
       </c>
-      <c r="V6" s="4" t="str">
+      <c r="V6" s="3" t="str">
         <v>2012-11-23T11:20</v>
       </c>
-      <c r="W6" s="4">
+      <c r="W6" s="3">
         <v>-7</v>
       </c>
-      <c r="X6" s="4" t="str">
-        <v/>
-      </c>
-      <c r="Y6" s="4">
+      <c r="X6" s="3" t="str">
+        <v/>
+      </c>
+      <c r="Y6" s="3">
         <v>2</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="str">
+      <c r="A7" s="3" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B7" s="4" t="str">
+      <c r="B7" s="3" t="str">
         <v>LB</v>
       </c>
-      <c r="C7" s="4" t="str">
+      <c r="C7" s="3" t="str">
         <v>CDISC001</v>
       </c>
-      <c r="D7" s="4">
+      <c r="D7" s="3">
         <v>2</v>
       </c>
-      <c r="E7" s="4" t="str">
+      <c r="E7" s="3" t="str">
         <v>ALP</v>
       </c>
-      <c r="F7" s="4" t="str">
+      <c r="F7" s="3" t="str">
         <v>Alkaline Phosphatase</v>
       </c>
-      <c r="G7" s="4" t="str">
+      <c r="G7" s="3" t="str">
         <v>CHEMISTRY</v>
       </c>
-      <c r="H7" s="4" t="str">
+      <c r="H7" s="3">
         <v>93</v>
       </c>
-      <c r="I7" s="4" t="str">
+      <c r="I7" s="3" t="str">
         <v>U/L</v>
       </c>
-      <c r="J7" s="4" t="str">
+      <c r="J7" s="3">
         <v>35</v>
       </c>
-      <c r="K7" s="4" t="str">
+      <c r="K7" s="3">
         <v>115</v>
       </c>
-      <c r="L7" s="4" t="str">
+      <c r="L7" s="3">
         <v>93</v>
       </c>
-      <c r="M7" s="4">
+      <c r="M7" s="3">
         <v>93</v>
       </c>
-      <c r="N7" s="4" t="str">
+      <c r="N7" s="3" t="str">
         <v>U/L</v>
       </c>
-      <c r="O7" s="4">
+      <c r="O7" s="3">
         <v>35</v>
       </c>
-      <c r="P7" s="4">
+      <c r="P7" s="3">
         <v>115</v>
       </c>
-      <c r="Q7" s="4" t="str">
+      <c r="Q7" s="3" t="str">
         <v>NORMAL</v>
       </c>
-      <c r="R7" s="4" t="str">
+      <c r="R7" s="3" t="str">
         <v>Y</v>
       </c>
-      <c r="S7" s="4">
+      <c r="S7" s="3">
         <v>1</v>
       </c>
-      <c r="T7" s="4" t="str">
+      <c r="T7" s="3" t="str">
         <v>SCREENING 1</v>
       </c>
-      <c r="U7" s="4" t="str">
+      <c r="U7" s="3" t="str">
         <v>SCREENING</v>
       </c>
-      <c r="V7" s="4" t="str">
+      <c r="V7" s="3" t="str">
         <v>2012-11-23T11:20</v>
       </c>
-      <c r="W7" s="4">
+      <c r="W7" s="3">
         <v>-7</v>
       </c>
-      <c r="X7" s="4" t="str">
-        <v/>
-      </c>
-      <c r="Y7" s="4" t="str">
+      <c r="X7" s="3" t="str">
+        <v/>
+      </c>
+      <c r="Y7" s="3" t="str">
         <v>Grade II</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="str">
+      <c r="A8" s="3" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B8" s="4" t="str">
+      <c r="B8" s="3" t="str">
         <v>LB</v>
       </c>
-      <c r="C8" s="4" t="str">
+      <c r="C8" s="3" t="str">
         <v>CDISC002</v>
       </c>
-      <c r="D8" s="4">
+      <c r="D8" s="3">
         <v>1</v>
       </c>
-      <c r="E8" s="4" t="str">
+      <c r="E8" s="3" t="str">
         <v>ALB</v>
       </c>
-      <c r="F8" s="4" t="str">
+      <c r="F8" s="3" t="str">
         <v>Albumin</v>
       </c>
-      <c r="G8" s="4" t="str">
+      <c r="G8" s="3" t="str">
         <v>CHEMISTRY</v>
       </c>
-      <c r="H8" s="4" t="str">
+      <c r="H8" s="3">
         <v>3.9</v>
       </c>
-      <c r="I8" s="4" t="str">
+      <c r="I8" s="3" t="str">
         <v>g/dL</v>
       </c>
-      <c r="J8" s="4" t="str">
+      <c r="J8" s="3">
         <v>3.5</v>
       </c>
-      <c r="K8" s="4" t="str">
+      <c r="K8" s="3">
         <v>4.6</v>
       </c>
-      <c r="L8" s="4" t="str">
+      <c r="L8" s="3">
         <v>39</v>
       </c>
-      <c r="M8" s="4">
+      <c r="M8" s="3">
         <v>39</v>
       </c>
-      <c r="N8" s="4" t="str">
+      <c r="N8" s="3" t="str">
         <v>g/L</v>
       </c>
-      <c r="O8" s="4">
+      <c r="O8" s="3">
         <v>35</v>
       </c>
-      <c r="P8" s="4">
+      <c r="P8" s="3">
         <v>46</v>
       </c>
-      <c r="Q8" s="4" t="str">
+      <c r="Q8" s="3" t="str">
         <v>NORMAL</v>
       </c>
-      <c r="R8" s="4" t="str">
+      <c r="R8" s="3" t="str">
         <v>Y</v>
       </c>
-      <c r="S8" s="4">
+      <c r="S8" s="3">
         <v>1</v>
       </c>
-      <c r="T8" s="4" t="str">
+      <c r="T8" s="3" t="str">
         <v>SCREENING 1</v>
       </c>
-      <c r="U8" s="4" t="str">
+      <c r="U8" s="3" t="str">
         <v>SCREENING</v>
       </c>
-      <c r="V8" s="4" t="str">
+      <c r="V8" s="3" t="str">
         <v>2012-11-23T11:20</v>
       </c>
-      <c r="W8" s="4">
+      <c r="W8" s="3">
         <v>-7</v>
       </c>
-      <c r="X8" s="4" t="str">
-        <v/>
-      </c>
-      <c r="Y8" s="4">
+      <c r="X8" s="3" t="str">
+        <v/>
+      </c>
+      <c r="Y8" s="3">
         <v>4</v>
       </c>
     </row>

</xml_diff>